<commit_message>
Pruebas Unitarias y de Caja blanca hechas
</commit_message>
<xml_diff>
--- a/Proyecto/docs/Pruebas de Caja Negra_Blanca/Plan de Pruebas Unitarias.xlsx
+++ b/Proyecto/docs/Pruebas de Caja Negra_Blanca/Plan de Pruebas Unitarias.xlsx
@@ -1,20 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/01f32f4e8c9e178e/Desktop/Analisis y Diseño/36289_AnalisisYDisenoDeSistemas/Proyecto/docs/Pruebas de Caja Negra_Blanca/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="226" documentId="11_C1C121B5557920B4F162870EFEB730A5709D5206" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7E1A714-4D12-4162-B5EA-F821E6A23D74}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Usuario" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Producto" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Venta" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="MetodoPago" sheetId="4" r:id="rId8"/>
+    <sheet name="Usuario" sheetId="1" r:id="rId1"/>
+    <sheet name="Cliente" sheetId="5" r:id="rId2"/>
+    <sheet name="Producto" sheetId="2" r:id="rId3"/>
+    <sheet name="Venta" sheetId="3" r:id="rId4"/>
+    <sheet name="MetodoPago" sheetId="4" r:id="rId5"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="622" uniqueCount="122">
   <si>
     <t>Caso de Éxito</t>
   </si>
@@ -64,9 +74,6 @@
     <t>No se guarda el resultado</t>
   </si>
   <si>
-    <t>andres1234!¿?&amp;(Muchos caracteres)</t>
-  </si>
-  <si>
     <t>11111andres1111, joshua222$$$$</t>
   </si>
   <si>
@@ -266,49 +273,164 @@
   </si>
   <si>
     <t>GetMonto(monto)</t>
+  </si>
+  <si>
+    <t>UsuarioConsultado</t>
+  </si>
+  <si>
+    <t>GetContraseña(contraseña)</t>
+  </si>
+  <si>
+    <t>GetIdTipoUsuario(idTipoUsuario)</t>
+  </si>
+  <si>
+    <t>andres1234!¿?&amp;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">andres1234!¿?&amp; </t>
+  </si>
+  <si>
+    <t>Se muestra el resultado</t>
+  </si>
+  <si>
+    <t>No se muestra el resultado</t>
+  </si>
+  <si>
+    <t>Se elimina el usuario</t>
+  </si>
+  <si>
+    <t>UsuarioEliminado</t>
+  </si>
+  <si>
+    <t>No se elimina el usuario</t>
+  </si>
+  <si>
+    <t>UsuarioModificado</t>
+  </si>
+  <si>
+    <t>AndresFabara, JoshuaOsorio</t>
+  </si>
+  <si>
+    <t>UpdateNombre(nombre)</t>
+  </si>
+  <si>
+    <t>UpdateContraseña(contraseña)</t>
+  </si>
+  <si>
+    <t>Andres123, Joshua987</t>
+  </si>
+  <si>
+    <t>123AndresEduardo987?¿¨^*Ç</t>
+  </si>
+  <si>
+    <t>ClienteRegistrado</t>
+  </si>
+  <si>
+    <t>ClienteConsultado</t>
+  </si>
+  <si>
+    <t>ClienteModificado</t>
+  </si>
+  <si>
+    <t>ClienteEliminado</t>
+  </si>
+  <si>
+    <t>SetTelefono(telefono)</t>
+  </si>
+  <si>
+    <t>SetApellido(apellido)</t>
+  </si>
+  <si>
+    <t>Fabara, Osorio</t>
+  </si>
+  <si>
+    <t>6649876543, 6641234567</t>
+  </si>
+  <si>
+    <t>and1234567, 66412345678</t>
+  </si>
+  <si>
+    <t>GetApellido(apellido)</t>
+  </si>
+  <si>
+    <t>GetTelefono(telefono)</t>
+  </si>
+  <si>
+    <t>UpdateApellido(apellido)</t>
+  </si>
+  <si>
+    <t>UpdateTelefono(telefono)</t>
+  </si>
+  <si>
+    <t>DeleteIdTipoUsuario(idTipoUsuario)</t>
+  </si>
+  <si>
+    <t>AndresEduardo, Joshua</t>
+  </si>
+  <si>
+    <t>Caicedo, Osorio</t>
+  </si>
+  <si>
+    <t>Caicedo123, Osorio 987</t>
+  </si>
+  <si>
+    <t>DeleteIdCliente(idCliente)</t>
+  </si>
+  <si>
+    <t>MetodoPagoEliminado</t>
+  </si>
+  <si>
+    <t>DeleteIdMetodoPago(idMetodoPago)</t>
+  </si>
+  <si>
+    <t>UpdateMonto(monto)</t>
+  </si>
+  <si>
+    <t>Efectivo, Tarjeta</t>
+  </si>
+  <si>
+    <t>2500.80</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy h:mm"/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="5">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="&quot;Aptos Narrow&quot;"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="&quot;Aptos Narrow&quot;"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -328,19 +450,39 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFEA8C2E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FF8ED973"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
-    <border/>
+  <borders count="11">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -355,6 +497,7 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -363,112 +506,157 @@
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
+      <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
+      <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="30">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="22" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="2" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="2" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="3" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="2" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="2" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="3" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -658,24 +846,27 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="B2:F41"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="16.25"/>
-    <col customWidth="1" min="3" max="3" width="24.25"/>
-    <col customWidth="1" min="4" max="4" width="29.88"/>
-    <col customWidth="1" min="5" max="5" width="33.25"/>
-    <col customWidth="1" min="6" max="6" width="25.0"/>
+    <col min="2" max="2" width="21.5703125" customWidth="1"/>
+    <col min="3" max="3" width="24.28515625" customWidth="1"/>
+    <col min="4" max="4" width="34.140625" customWidth="1"/>
+    <col min="5" max="5" width="37.140625" customWidth="1"/>
+    <col min="6" max="6" width="26.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2">
+    <row r="2" spans="2:6">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -692,7 +883,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="2:6">
       <c r="B3" s="3"/>
       <c r="C3" s="2" t="s">
         <v>5</v>
@@ -707,7 +898,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="2:6">
       <c r="B4" s="3"/>
       <c r="C4" s="2" t="s">
         <v>5</v>
@@ -722,7 +913,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="2:6">
       <c r="B5" s="3"/>
       <c r="C5" s="2" t="s">
         <v>5</v>
@@ -737,21 +928,21 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="2:6">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7">
+    <row r="7" spans="2:6">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8">
+    <row r="8" spans="2:6">
       <c r="B8" s="4" t="s">
         <v>13</v>
       </c>
@@ -768,7 +959,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="2:6">
       <c r="B9" s="3"/>
       <c r="C9" s="5" t="s">
         <v>5</v>
@@ -783,7 +974,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="2:6">
       <c r="B10" s="3"/>
       <c r="C10" s="5" t="s">
         <v>5</v>
@@ -792,13 +983,13 @@
         <v>9</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>16</v>
+        <v>87</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="2:6">
       <c r="B11" s="3"/>
       <c r="C11" s="5" t="s">
         <v>5</v>
@@ -807,32 +998,940 @@
         <v>11</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>15</v>
       </c>
     </row>
+    <row r="14" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B14" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B15" s="3"/>
+      <c r="C15" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B16" s="3"/>
+      <c r="C16" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B17" s="3"/>
+      <c r="C17" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+    </row>
+    <row r="19" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+    </row>
+    <row r="20" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B20" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B21" s="3"/>
+      <c r="C21" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B22" s="3"/>
+      <c r="C22" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B23" s="3"/>
+      <c r="C23" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="D23" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="E23" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="F23" s="21" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B24" s="3"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="18"/>
+    </row>
+    <row r="26" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B26" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E26" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="F26" s="22" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B27" s="3"/>
+      <c r="C27" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="D27" s="28" t="s">
+        <v>95</v>
+      </c>
+      <c r="E27" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="F27" s="24" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B28" s="3"/>
+      <c r="C28" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="D28" s="29" t="s">
+        <v>96</v>
+      </c>
+      <c r="E28" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="F28" s="24" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B29" s="3"/>
+      <c r="C29" s="23"/>
+      <c r="D29" s="23"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="23"/>
+    </row>
+    <row r="30" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+    </row>
+    <row r="31" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+    </row>
+    <row r="32" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B32" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E32" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="F32" s="20" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B33" s="3"/>
+      <c r="C33" s="19" t="s">
+        <v>93</v>
+      </c>
+      <c r="D33" s="26" t="s">
+        <v>95</v>
+      </c>
+      <c r="E33" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="F33" s="25" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B34" s="3"/>
+      <c r="C34" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="D34" s="27" t="s">
+        <v>96</v>
+      </c>
+      <c r="E34" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="F34" s="25" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B35" s="3"/>
+      <c r="C35" s="18"/>
+      <c r="D35" s="18"/>
+      <c r="E35" s="18"/>
+      <c r="F35" s="18"/>
+    </row>
+    <row r="37" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B37" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B38" s="3"/>
+      <c r="C38" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B40" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="41" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B41" s="3"/>
+      <c r="C41" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>92</v>
+      </c>
+    </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FF8663A-C997-4B4B-B81A-B32C9EEC73B6}">
+  <dimension ref="B4:F49"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75"/>
+  <cols>
+    <col min="2" max="2" width="27.5703125" customWidth="1"/>
+    <col min="3" max="3" width="26.7109375" customWidth="1"/>
+    <col min="4" max="4" width="40.5703125" customWidth="1"/>
+    <col min="5" max="5" width="35.7109375" customWidth="1"/>
+    <col min="6" max="6" width="29.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="2:6" ht="14.25">
+      <c r="B4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" ht="14.25">
+      <c r="B5" s="3"/>
+      <c r="C5" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" ht="14.25">
+      <c r="B6" s="3"/>
+      <c r="C6" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" ht="14.25">
+      <c r="B7" s="3"/>
+      <c r="C7" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" ht="14.25">
+      <c r="B8" s="3"/>
+      <c r="C8" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" ht="14.25">
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+    </row>
+    <row r="10" spans="2:6" ht="14.25">
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+    </row>
+    <row r="11" spans="2:6" ht="14.25">
+      <c r="B11" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" ht="14.25">
+      <c r="B12" s="3"/>
+      <c r="C12" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" ht="14.25">
+      <c r="B13" s="3"/>
+      <c r="C13" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" ht="14.25">
+      <c r="B14" s="3"/>
+      <c r="C14" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" ht="14.25">
+      <c r="B15" s="3"/>
+      <c r="C15" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" ht="14.25">
+      <c r="B18" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" ht="14.25">
+      <c r="B19" s="3"/>
+      <c r="C19" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" ht="14.25">
+      <c r="B20" s="3"/>
+      <c r="C20" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" ht="14.25">
+      <c r="B21" s="3"/>
+      <c r="C21" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" ht="14.25">
+      <c r="B22" s="3"/>
+      <c r="C22" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" ht="14.25">
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+    </row>
+    <row r="24" spans="2:6" ht="14.25">
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+    </row>
+    <row r="25" spans="2:6" ht="14.25">
+      <c r="B25" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C25" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="E25" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="F25" s="20" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" ht="14.25">
+      <c r="B26" s="3"/>
+      <c r="C26" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="D26" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="E26" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" ht="14.25">
+      <c r="B27" s="3"/>
+      <c r="C27" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="D27" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="E27" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" ht="14.25">
+      <c r="B28" s="3"/>
+      <c r="C28" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="D28" s="25" t="s">
+        <v>109</v>
+      </c>
+      <c r="E28" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="F28" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" ht="14.25">
+      <c r="B29" s="3"/>
+      <c r="C29" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="D29" s="25" t="s">
+        <v>59</v>
+      </c>
+      <c r="E29" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="F29" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" ht="14.25">
+      <c r="B30" s="3"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
+    </row>
+    <row r="32" spans="2:6" ht="14.25">
+      <c r="B32" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C32" s="22" t="s">
+        <v>1</v>
+      </c>
+      <c r="D32" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="E32" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="F32" s="22" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" ht="14.25">
+      <c r="B33" s="3"/>
+      <c r="C33" s="24" t="s">
+        <v>101</v>
+      </c>
+      <c r="D33" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="E33" s="24" t="s">
+        <v>113</v>
+      </c>
+      <c r="F33" s="24" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" ht="14.25">
+      <c r="B34" s="3"/>
+      <c r="C34" s="24" t="s">
+        <v>101</v>
+      </c>
+      <c r="D34" s="24" t="s">
+        <v>110</v>
+      </c>
+      <c r="E34" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="F34" s="24" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" ht="14.25">
+      <c r="B35" s="3"/>
+      <c r="C35" s="24" t="s">
+        <v>101</v>
+      </c>
+      <c r="D35" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="E35" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="F35" s="24" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" ht="14.25">
+      <c r="B36" s="3"/>
+      <c r="C36" s="23"/>
+      <c r="D36" s="23"/>
+      <c r="E36" s="23"/>
+      <c r="F36" s="23"/>
+    </row>
+    <row r="37" spans="2:6" ht="14.25">
+      <c r="B37" s="3"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
+    </row>
+    <row r="38" spans="2:6" ht="14.25">
+      <c r="B38" s="3"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+    </row>
+    <row r="39" spans="2:6" ht="14.25">
+      <c r="B39" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C39" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="D39" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="E39" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="F39" s="20" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6" ht="14.25">
+      <c r="B40" s="3"/>
+      <c r="C40" s="25" t="s">
+        <v>101</v>
+      </c>
+      <c r="D40" s="25" t="s">
+        <v>95</v>
+      </c>
+      <c r="E40" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="F40" s="25" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="41" spans="2:6" ht="14.25">
+      <c r="B41" s="3"/>
+      <c r="C41" s="25" t="s">
+        <v>101</v>
+      </c>
+      <c r="D41" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="E41" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="F41" s="25" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="42" spans="2:6" ht="14.25">
+      <c r="B42" s="3"/>
+      <c r="C42" s="25" t="s">
+        <v>101</v>
+      </c>
+      <c r="D42" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="E42" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="F42" s="25" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="43" spans="2:6" ht="14.25">
+      <c r="B43" s="3"/>
+      <c r="C43" s="18"/>
+      <c r="D43" s="18"/>
+      <c r="E43" s="18"/>
+      <c r="F43" s="18"/>
+    </row>
+    <row r="45" spans="2:6" ht="14.25">
+      <c r="B45" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="46" spans="2:6" ht="14.25">
+      <c r="B46" s="3"/>
+      <c r="C46" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="48" spans="2:6" ht="14.25">
+      <c r="B48" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49" spans="2:6" ht="14.25">
+      <c r="B49" s="3"/>
+      <c r="C49" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F49" s="6" t="s">
+        <v>92</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="B2:F43"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="17.38"/>
-    <col customWidth="1" min="3" max="3" width="31.5"/>
-    <col customWidth="1" min="4" max="4" width="44.88"/>
-    <col customWidth="1" min="5" max="5" width="28.38"/>
-    <col customWidth="1" min="6" max="6" width="26.75"/>
+    <col min="2" max="2" width="17.42578125" customWidth="1"/>
+    <col min="3" max="3" width="31.42578125" customWidth="1"/>
+    <col min="4" max="4" width="44.85546875" customWidth="1"/>
+    <col min="5" max="5" width="28.42578125" customWidth="1"/>
+    <col min="6" max="6" width="26.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2">
+    <row r="2" spans="2:6">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -849,43 +1948,43 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="2:6">
       <c r="B3" s="3"/>
       <c r="C3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>20</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="2:6">
       <c r="B4" s="3"/>
       <c r="C4" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>22</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="2:6">
       <c r="B5" s="3"/>
       <c r="C5" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>12</v>
@@ -894,21 +1993,21 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="2:6">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7">
+    <row r="7" spans="2:6">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8">
+    <row r="8" spans="2:6">
       <c r="B8" s="4" t="s">
         <v>13</v>
       </c>
@@ -925,13 +2024,13 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="2:6">
       <c r="B9" s="3"/>
       <c r="C9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>18</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>19</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>14</v>
@@ -940,58 +2039,58 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="2:6">
       <c r="B10" s="3"/>
       <c r="C10" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="2:6">
       <c r="B11" s="3"/>
       <c r="C11" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="2:6">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
     </row>
-    <row r="13">
+    <row r="13" spans="2:6">
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
-    <row r="14">
+    <row r="14" spans="2:6">
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
     </row>
-    <row r="15">
+    <row r="15" spans="2:6">
       <c r="B15" s="1" t="s">
         <v>0</v>
       </c>
@@ -1008,66 +2107,66 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="2:6">
       <c r="B16" s="3"/>
       <c r="C16" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="E16" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="17">
+    </row>
+    <row r="17" spans="2:6">
       <c r="B17" s="3"/>
       <c r="C17" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D17" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>30</v>
-      </c>
       <c r="F17" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="18">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6">
       <c r="B18" s="3"/>
       <c r="C18" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="19">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6">
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
-    <row r="20">
+    <row r="20" spans="2:6">
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
-    <row r="21">
+    <row r="21" spans="2:6">
       <c r="B21" s="4" t="s">
         <v>13</v>
       </c>
@@ -1084,66 +2183,66 @@
         <v>4</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="2:6">
       <c r="B22" s="3"/>
       <c r="C22" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D22" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="23">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6">
       <c r="B23" s="3"/>
       <c r="C23" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="24">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6">
       <c r="B24" s="3"/>
       <c r="C24" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D24" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F24" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="E24" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F24" s="6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="25">
+    </row>
+    <row r="25" spans="2:6">
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
     </row>
-    <row r="26">
+    <row r="26" spans="2:6">
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
     </row>
-    <row r="27">
+    <row r="27" spans="2:6">
       <c r="B27" s="1" t="s">
         <v>0</v>
       </c>
@@ -1160,58 +2259,58 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="2:6">
       <c r="B28" s="3"/>
       <c r="C28" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="E28" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E28" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="F28" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="29">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6">
       <c r="B29" s="3"/>
       <c r="C29" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="30">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6">
       <c r="B30" s="7"/>
       <c r="C30" s="8"/>
       <c r="D30" s="8"/>
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
     </row>
-    <row r="31">
+    <row r="31" spans="2:6">
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
     </row>
-    <row r="32">
+    <row r="32" spans="2:6">
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
     </row>
-    <row r="33">
+    <row r="33" spans="2:6">
       <c r="B33" s="4" t="s">
         <v>13</v>
       </c>
@@ -1228,51 +2327,51 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="2:6">
       <c r="B34" s="3"/>
       <c r="C34" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D34" s="4" t="s">
         <v>33</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>34</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6">
       <c r="B35" s="3"/>
       <c r="C35" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="36">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6">
       <c r="B36" s="7"/>
       <c r="C36" s="9"/>
       <c r="D36" s="9"/>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
     </row>
-    <row r="37">
+    <row r="37" spans="2:6">
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
     </row>
-    <row r="38">
+    <row r="38" spans="2:6">
       <c r="B38" s="1" t="s">
         <v>0</v>
       </c>
@@ -1289,36 +2388,36 @@
         <v>4</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="2:6">
       <c r="B39" s="3"/>
       <c r="C39" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D39" s="2" t="s">
+      <c r="E39" s="10">
+        <v>12345678</v>
+      </c>
+      <c r="F39" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E39" s="10">
-        <v>1.2345678E7</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="40">
+    </row>
+    <row r="40" spans="2:6">
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
     </row>
-    <row r="41">
+    <row r="41" spans="2:6">
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
     </row>
-    <row r="42">
+    <row r="42" spans="2:6">
       <c r="B42" s="4" t="s">
         <v>13</v>
       </c>
@@ -1335,41 +2434,42 @@
         <v>4</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="2:6">
       <c r="B43" s="3"/>
       <c r="C43" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E43" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="F43" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F43" s="6" t="s">
-        <v>41</v>
-      </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="B2:F49"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="19.0"/>
-    <col customWidth="1" min="3" max="3" width="25.5"/>
-    <col customWidth="1" min="4" max="4" width="45.5"/>
-    <col customWidth="1" min="5" max="5" width="22.38"/>
-    <col customWidth="1" min="6" max="6" width="26.75"/>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="3" max="3" width="25.42578125" customWidth="1"/>
+    <col min="4" max="4" width="45.42578125" customWidth="1"/>
+    <col min="5" max="5" width="22.42578125" customWidth="1"/>
+    <col min="6" max="6" width="26.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2">
+    <row r="2" spans="2:6">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1386,28 +2486,28 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="2:6">
       <c r="B3" s="3"/>
       <c r="C3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>44</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="2:6">
       <c r="B4" s="3"/>
       <c r="C4" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E4" s="11">
         <v>46198.666666666664</v>
@@ -1416,13 +2516,13 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="2:6">
       <c r="B5" s="3"/>
       <c r="C5" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>12</v>
@@ -1431,13 +2531,13 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="2:6">
       <c r="B6" s="3"/>
       <c r="C6" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>12</v>
@@ -1446,13 +2546,13 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="2:6">
       <c r="B7" s="3"/>
       <c r="C7" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>12</v>
@@ -1461,13 +2561,13 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="2:6">
       <c r="B8" s="3"/>
       <c r="C8" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>12</v>
@@ -1476,14 +2576,14 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="2:6">
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
     </row>
-    <row r="10">
+    <row r="10" spans="2:6">
       <c r="B10" s="4" t="s">
         <v>13</v>
       </c>
@@ -1500,13 +2600,13 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="2:6">
       <c r="B11" s="3"/>
       <c r="C11" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>42</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>43</v>
       </c>
       <c r="E11" s="12">
         <v>2350.6</v>
@@ -1515,89 +2615,89 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="2:6">
       <c r="B12" s="3"/>
       <c r="C12" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="2:6">
       <c r="B13" s="3"/>
       <c r="C13" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="2:6">
       <c r="B14" s="3"/>
       <c r="C14" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="2:6">
       <c r="B15" s="3"/>
       <c r="C15" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="2:6">
       <c r="B16" s="3"/>
       <c r="C16" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="2:6">
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
     </row>
-    <row r="18">
+    <row r="18" spans="2:6">
       <c r="B18" s="1" t="s">
         <v>0</v>
       </c>
@@ -1614,104 +2714,104 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="2:6">
       <c r="B19" s="3"/>
       <c r="C19" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>56</v>
-      </c>
       <c r="E19" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="20">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6">
       <c r="B20" s="3"/>
       <c r="C20" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E20" s="11">
         <v>46198.666666666664</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="21">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6">
       <c r="B21" s="3"/>
       <c r="C21" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="22">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6">
       <c r="B22" s="3"/>
       <c r="C22" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="23">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6">
       <c r="B23" s="3"/>
       <c r="C23" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="24">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6">
       <c r="B24" s="3"/>
       <c r="C24" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6">
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
     </row>
-    <row r="26">
+    <row r="26" spans="2:6">
       <c r="B26" s="4" t="s">
         <v>13</v>
       </c>
@@ -1728,111 +2828,111 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="2:6">
       <c r="B27" s="3"/>
       <c r="C27" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D27" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="E27" s="12">
         <v>2350.65</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="28">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6">
       <c r="B28" s="3"/>
       <c r="C28" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="29">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6">
       <c r="B29" s="3"/>
       <c r="C29" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="30">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6">
       <c r="B30" s="3"/>
       <c r="C30" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="31">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6">
       <c r="B31" s="3"/>
       <c r="C31" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="32">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6">
       <c r="B32" s="3"/>
       <c r="C32" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="33">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6">
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
     </row>
-    <row r="34">
+    <row r="34" spans="2:6">
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
     </row>
-    <row r="35">
+    <row r="35" spans="2:6">
       <c r="B35" s="1" t="s">
         <v>0</v>
       </c>
@@ -1849,44 +2949,44 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="2:6">
       <c r="B36" s="3"/>
       <c r="C36" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="E36" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E36" s="2" t="s">
+      <c r="F36" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="F36" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="37">
+    </row>
+    <row r="37" spans="2:6">
       <c r="B37" s="3"/>
       <c r="C37" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E37" s="11">
         <v>46228.75</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="38">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6">
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
-    <row r="39">
+    <row r="39" spans="2:6">
       <c r="B39" s="4" t="s">
         <v>13</v>
       </c>
@@ -1903,51 +3003,51 @@
         <v>4</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="2:6">
       <c r="B40" s="3"/>
       <c r="C40" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D40" s="4" t="s">
         <v>63</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>64</v>
       </c>
       <c r="E40" s="12">
         <v>2350.85</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="41">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="41" spans="2:6">
       <c r="B41" s="3"/>
       <c r="C41" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D41" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F41" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="E41" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="F41" s="6" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="42">
+    </row>
+    <row r="42" spans="2:6">
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
     </row>
-    <row r="43">
+    <row r="43" spans="2:6">
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
     </row>
-    <row r="44">
+    <row r="44" spans="2:6">
       <c r="B44" s="1" t="s">
         <v>0</v>
       </c>
@@ -1964,36 +3064,36 @@
         <v>4</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="2:6">
       <c r="B45" s="3"/>
       <c r="C45" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="D45" s="2" t="s">
-        <v>71</v>
-      </c>
       <c r="E45" s="10">
-        <v>1.2345678E7</v>
+        <v>12345678</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="46">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="46" spans="2:6">
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
     </row>
-    <row r="47">
+    <row r="47" spans="2:6">
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
     </row>
-    <row r="48">
+    <row r="48" spans="2:6">
       <c r="B48" s="4" t="s">
         <v>13</v>
       </c>
@@ -2010,41 +3110,42 @@
         <v>4</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="2:6">
       <c r="B49" s="3"/>
       <c r="C49" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D49" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="D49" s="4" t="s">
-        <v>71</v>
-      </c>
       <c r="E49" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="F49" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F49" s="6" t="s">
-        <v>41</v>
-      </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="B2:H36"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="17.13"/>
-    <col customWidth="1" min="3" max="3" width="30.75"/>
-    <col customWidth="1" min="4" max="4" width="38.25"/>
-    <col customWidth="1" min="5" max="5" width="22.5"/>
-    <col customWidth="1" min="6" max="6" width="25.38"/>
+    <col min="2" max="2" width="17.140625" customWidth="1"/>
+    <col min="3" max="3" width="30.7109375" customWidth="1"/>
+    <col min="4" max="4" width="38.28515625" customWidth="1"/>
+    <col min="5" max="5" width="22.42578125" customWidth="1"/>
+    <col min="6" max="6" width="25.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2">
+    <row r="2" spans="2:8">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2061,71 +3162,71 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="2:8">
       <c r="B3" s="3"/>
       <c r="C3" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8">
       <c r="B4" s="3"/>
       <c r="C4" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8">
       <c r="B5" s="3"/>
       <c r="C5" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E5" s="10">
-        <v>1.2345678E7</v>
+        <v>12345678</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
       <c r="H6" s="13" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8">
       <c r="B7" s="4" t="s">
         <v>13</v>
       </c>
@@ -2142,10 +3243,10 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="2:8">
       <c r="B8" s="3"/>
       <c r="C8" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>6</v>
@@ -2157,13 +3258,13 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="2:8">
       <c r="B9" s="3"/>
       <c r="C9" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E9" s="14">
         <v>2350.65</v>
@@ -2172,22 +3273,22 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="2:8">
       <c r="B10" s="3"/>
       <c r="C10" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="2:8">
       <c r="B12" s="1" t="s">
         <v>0</v>
       </c>
@@ -2204,59 +3305,59 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="2:8">
       <c r="B13" s="3"/>
       <c r="C13" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="D13" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="D13" s="15" t="s">
-        <v>82</v>
-      </c>
       <c r="E13" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="2:8">
       <c r="B14" s="3"/>
       <c r="C14" s="15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="2:8">
       <c r="B15" s="3"/>
       <c r="C15" s="15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E15" s="10">
-        <v>1.2345678E7</v>
+        <v>12345678</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="2:8">
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
     </row>
-    <row r="17">
+    <row r="17" spans="2:6">
       <c r="B17" s="4" t="s">
         <v>13</v>
       </c>
@@ -2273,13 +3374,13 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="2:6">
       <c r="B18" s="3"/>
       <c r="C18" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="D18" s="17" t="s">
         <v>81</v>
-      </c>
-      <c r="D18" s="17" t="s">
-        <v>82</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>14</v>
@@ -2288,13 +3389,13 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="2:6">
       <c r="B19" s="3"/>
       <c r="C19" s="16" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E19" s="14">
         <v>2350.65</v>
@@ -2303,22 +3404,194 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="2:6">
       <c r="B20" s="3"/>
       <c r="C20" s="16" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>15</v>
       </c>
     </row>
+    <row r="22" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B22" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B23" s="3"/>
+      <c r="C23" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B24" s="3"/>
+      <c r="C24" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B26" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B27" s="3"/>
+      <c r="C27" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="D27" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B28" s="3"/>
+      <c r="C28" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="D28" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="E28" s="14">
+        <v>2550.6950000000002</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B31" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B32" s="3"/>
+      <c r="C32" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E32" s="10">
+        <v>12345678</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+    </row>
+    <row r="34" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+    </row>
+    <row r="35" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B35" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" ht="15.75" customHeight="1">
+      <c r="B36" s="3"/>
+      <c r="C36" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>